<commit_message>
Catalog Hamilton Secondary Plan Land Use and PolicyPlanning service
</commit_message>
<xml_diff>
--- a/Spreadsheets/02-dataset-inventory-v4.xlsx
+++ b/Spreadsheets/02-dataset-inventory-v4.xlsx
@@ -27927,7 +27927,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>hamilton_zoning_ped_legacy</t>
+          <t>hamilton_secondary_plan_land_use</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -27937,7 +27937,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Hamilton Zoning PED_ZONING pre-Rural / council-approved</t>
+          <t>Hamilton Secondary Plan Land Use</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -27947,7 +27947,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/PED_ZONING_preRural_/FeatureServer/0</t>
+          <t>https://spatialsolutions.hamilton.ca/webgis/rest/services/General/PolicyPlanning/MapServer/6</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -27962,12 +27962,12 @@
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>full</t>
+          <t>partial</t>
         </is>
       </c>
       <c r="I85" t="inlineStr">
         <is>
-          <t>legacy / working zoning polygons</t>
+          <t>secondary plan land-use designation polygons</t>
         </is>
       </c>
       <c r="J85" t="inlineStr">
@@ -28007,17 +28007,17 @@
       </c>
       <c r="Q85" t="inlineStr">
         <is>
-          <t>9413 + 1872 (live REST 2026-10-17)</t>
+          <t>47212 polygons, 31 plans, 67 classes (live REST 2026-10-17)</t>
         </is>
       </c>
       <c r="R85" t="inlineStr">
         <is>
-          <t/>
+          <t>yes -- filter 4 retired plans | reconcile plan names to boundary layer | dissolve by designation</t>
         </is>
       </c>
       <c r="S85" t="inlineStr">
         <is>
-          <t/>
+          <t>filter | dissolve | polygon overlay</t>
         </is>
       </c>
       <c r="T85" t="inlineStr">
@@ -28027,12 +28027,12 @@
       </c>
       <c r="U85" t="inlineStr">
         <is>
-          <t/>
+          <t>not stated [no licence published on the service; not on open.hamilton.ca; recorded for provenance, HARD-RULES 6]</t>
         </is>
       </c>
       <c r="V85" t="inlineStr">
         <is>
-          <t>unclear</t>
+          <t>allowed_by_rule</t>
         </is>
       </c>
       <c r="W85" t="inlineStr">
@@ -28057,7 +28057,7 @@
       </c>
       <c r="AA85" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="AB85" t="inlineStr">
@@ -28082,12 +28082,12 @@
       </c>
       <c r="AF85" t="inlineStr">
         <is>
-          <t>constraint</t>
+          <t>enrich</t>
         </is>
       </c>
       <c r="AG85" t="inlineStr">
         <is>
-          <t/>
+          <t>enrich</t>
         </is>
       </c>
       <c r="AH85" t="inlineStr">
@@ -28107,7 +28107,7 @@
       </c>
       <c r="AK85" t="inlineStr">
         <is>
-          <t>Hamilton grouping analysis 2026-10-17</t>
+          <t>Hamilton OP designation source search 2026-10-17</t>
         </is>
       </c>
       <c r="AL85" t="inlineStr">
@@ -28172,7 +28172,7 @@
       </c>
       <c r="AX85" t="inlineStr">
         <is>
-          <t>A03. Unclear status vs hamilton_zoning_boundary; may be superseded [inferred]. COUNCAP_LDR sibling noted in grouping, URL not separately confirmed here. Evidence: live_rest.</t>
+          <t>Provisional OP designation source (secondary plan areas only). No public citywide UHOP Schedule E-1 / RHOP Schedule D layer exists; that remains a named gap. Last amended 2026-05-12. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY85" t="inlineStr">
@@ -28259,7 +28259,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>hamilton_parks</t>
+          <t>hamilton_zoning_ped_legacy</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -28269,7 +28269,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Hamilton Parks (Parks_OD)</t>
+          <t>Hamilton Zoning PED_ZONING pre-Rural / council-approved</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -28279,7 +28279,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/Parks_OD/FeatureServer/6</t>
+          <t>https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/PED_ZONING_preRural_/FeatureServer/0</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -28299,7 +28299,7 @@
       </c>
       <c r="I86" t="inlineStr">
         <is>
-          <t>municipal park polygons</t>
+          <t>legacy / working zoning polygons</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
@@ -28309,7 +28309,7 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>NAME | PARK_CLASS | ZONING_COD</t>
+          <t/>
         </is>
       </c>
       <c r="L86" t="inlineStr">
@@ -28339,7 +28339,7 @@
       </c>
       <c r="Q86" t="inlineStr">
         <is>
-          <t>633 polygons (live REST 2026-10-17)</t>
+          <t>9413 + 1872 (live REST 2026-10-17)</t>
         </is>
       </c>
       <c r="R86" t="inlineStr">
@@ -28389,7 +28389,7 @@
       </c>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="AB86" t="inlineStr">
@@ -28414,12 +28414,12 @@
       </c>
       <c r="AF86" t="inlineStr">
         <is>
-          <t>basemap</t>
+          <t>constraint</t>
         </is>
       </c>
       <c r="AG86" t="inlineStr">
         <is>
-          <t>basemap</t>
+          <t/>
         </is>
       </c>
       <c r="AH86" t="inlineStr">
@@ -28504,7 +28504,7 @@
       </c>
       <c r="AX86" t="inlineStr">
         <is>
-          <t>A04. Re-admitted from reviewed_not_relevant. Needed for the city-framed-by-nature first view. Evidence: live_rest.</t>
+          <t>A03. Unclear status vs hamilton_zoning_boundary; may be superseded [inferred]. COUNCAP_LDR sibling noted in grouping, URL not separately confirmed here. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY86" t="inlineStr">
@@ -28524,12 +28524,12 @@
       </c>
       <c r="BB86" t="inlineStr">
         <is>
-          <t>contextual_only</t>
+          <t/>
         </is>
       </c>
       <c r="BC86" t="inlineStr">
         <is>
-          <t>constraints</t>
+          <t>land_use</t>
         </is>
       </c>
       <c r="BD86" t="inlineStr">
@@ -28591,7 +28591,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>hamilton_trails</t>
+          <t>hamilton_parks</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -28601,7 +28601,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Hamilton Trails</t>
+          <t>Hamilton Parks (Parks_OD)</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -28611,7 +28611,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/Trails/FeatureServer/14</t>
+          <t>https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/Parks_OD/FeatureServer/6</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -28631,7 +28631,7 @@
       </c>
       <c r="I87" t="inlineStr">
         <is>
-          <t>trail lines</t>
+          <t>municipal park polygons</t>
         </is>
       </c>
       <c r="J87" t="inlineStr">
@@ -28641,7 +28641,7 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>TRAIL_NAME | BRUCE_TRAIL</t>
+          <t>NAME | PARK_CLASS | ZONING_COD</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
@@ -28671,7 +28671,7 @@
       </c>
       <c r="Q87" t="inlineStr">
         <is>
-          <t>3437 lines (live REST 2026-10-17)</t>
+          <t>633 polygons (live REST 2026-10-17)</t>
         </is>
       </c>
       <c r="R87" t="inlineStr">
@@ -28721,7 +28721,7 @@
       </c>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="AB87" t="inlineStr">
@@ -28751,7 +28751,7 @@
       </c>
       <c r="AG87" t="inlineStr">
         <is>
-          <t/>
+          <t>basemap</t>
         </is>
       </c>
       <c r="AH87" t="inlineStr">
@@ -28836,7 +28836,7 @@
       </c>
       <c r="AX87" t="inlineStr">
         <is>
-          <t>A05. Re-admitted from reviewed_not_relevant. Nature-frame P2. Evidence: live_rest.</t>
+          <t>A04. Re-admitted from reviewed_not_relevant. Needed for the city-framed-by-nature first view. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY87" t="inlineStr">
@@ -28861,7 +28861,7 @@
       </c>
       <c r="BC87" t="inlineStr">
         <is>
-          <t/>
+          <t>constraints</t>
         </is>
       </c>
       <c r="BD87" t="inlineStr">
@@ -28923,7 +28923,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>hamilton_wetlands</t>
+          <t>hamilton_trails</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -28933,17 +28933,17 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Hamilton Wetlands (City copy of provincial wetlands)</t>
+          <t>Hamilton Trails</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>City of Hamilton (from MNR)</t>
+          <t>City of Hamilton</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/Wetlands_COH_shp/FeatureServer/0</t>
+          <t>https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/Trails/FeatureServer/14</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -28963,7 +28963,7 @@
       </c>
       <c r="I88" t="inlineStr">
         <is>
-          <t>wetland polygons</t>
+          <t>trail lines</t>
         </is>
       </c>
       <c r="J88" t="inlineStr">
@@ -28973,7 +28973,7 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t/>
+          <t>TRAIL_NAME | BRUCE_TRAIL</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
@@ -29003,7 +29003,7 @@
       </c>
       <c r="Q88" t="inlineStr">
         <is>
-          <t>2693 polygons (live REST 2026-10-17)</t>
+          <t>3437 lines (live REST 2026-10-17)</t>
         </is>
       </c>
       <c r="R88" t="inlineStr">
@@ -29078,7 +29078,7 @@
       </c>
       <c r="AF88" t="inlineStr">
         <is>
-          <t>constraint</t>
+          <t>basemap</t>
         </is>
       </c>
       <c r="AG88" t="inlineStr">
@@ -29168,7 +29168,7 @@
       </c>
       <c r="AX88" t="inlineStr">
         <is>
-          <t>A06. Prefer over LIO wetlands clip inside Hamilton. Evidence: live_rest.</t>
+          <t>A05. Re-admitted from reviewed_not_relevant. Nature-frame P2. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY88" t="inlineStr">
@@ -29188,12 +29188,12 @@
       </c>
       <c r="BB88" t="inlineStr">
         <is>
-          <t/>
+          <t>contextual_only</t>
         </is>
       </c>
       <c r="BC88" t="inlineStr">
         <is>
-          <t>constraints</t>
+          <t/>
         </is>
       </c>
       <c r="BD88" t="inlineStr">
@@ -29255,7 +29255,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>hamilton_conservation_authority_areas</t>
+          <t>hamilton_wetlands</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -29265,24 +29265,24 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Hamilton conservation authority watershed areas (dissolved)</t>
+          <t>Hamilton Wetlands (City copy of provincial wetlands)</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
+          <t>City of Hamilton (from MNR)</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/Wetlands_COH_shp/FeatureServer/0</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
           <t>City of Hamilton</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/Hamilton_Conservation_Watersheds_Dissolved/FeatureServer/0 | https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/Conservation_Halton_Conservation_Watersheds_Dissolved/FeatureServer/0 | https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/Niagara_Conservation_Watersheds_Dissolved/FeatureServer/0 | https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/GRCA_Conservation_Watersheds_Dissolved/FeatureServer/0</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>City of Hamilton</t>
-        </is>
-      </c>
       <c r="G89" t="inlineStr">
         <is>
           <t>ON-Hamilton</t>
@@ -29295,7 +29295,7 @@
       </c>
       <c r="I89" t="inlineStr">
         <is>
-          <t>dissolved CA watershed polygons</t>
+          <t>wetland polygons</t>
         </is>
       </c>
       <c r="J89" t="inlineStr">
@@ -29305,7 +29305,7 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>CONSERVATION_AUTHORITY</t>
+          <t/>
         </is>
       </c>
       <c r="L89" t="inlineStr">
@@ -29335,7 +29335,7 @@
       </c>
       <c r="Q89" t="inlineStr">
         <is>
-          <t>4 polygons, 1 per CA (live REST 2026-10-17)</t>
+          <t>2693 polygons (live REST 2026-10-17)</t>
         </is>
       </c>
       <c r="R89" t="inlineStr">
@@ -29385,7 +29385,7 @@
       </c>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="AB89" t="inlineStr">
@@ -29500,7 +29500,7 @@
       </c>
       <c r="AX89" t="inlineStr">
         <is>
-          <t>A07. Four URLs expanded from the grouping template [inferred expansion]. Names the regulating CA so CH/GRCA refusals stay honest. Evidence: live_rest.</t>
+          <t>A06. Prefer over LIO wetlands clip inside Hamilton. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY89" t="inlineStr">
@@ -29587,7 +29587,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>hamilton_subwatersheds</t>
+          <t>hamilton_conservation_authority_areas</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -29597,7 +29597,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Hamilton HCA / NPCA subwatersheds and watershed grades</t>
+          <t>Hamilton conservation authority watershed areas (dissolved)</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -29607,7 +29607,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/HCA_Subwatersheds/FeatureServer | https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/NPCA_Subwatersheds/FeatureServer | https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/Watershed_Grades/FeatureServer</t>
+          <t>https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/Hamilton_Conservation_Watersheds_Dissolved/FeatureServer/0 | https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/Conservation_Halton_Conservation_Watersheds_Dissolved/FeatureServer/0 | https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/Niagara_Conservation_Watersheds_Dissolved/FeatureServer/0 | https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/GRCA_Conservation_Watersheds_Dissolved/FeatureServer/0</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -29627,7 +29627,7 @@
       </c>
       <c r="I90" t="inlineStr">
         <is>
-          <t>subwatershed polygons</t>
+          <t>dissolved CA watershed polygons</t>
         </is>
       </c>
       <c r="J90" t="inlineStr">
@@ -29637,7 +29637,7 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t/>
+          <t>CONSERVATION_AUTHORITY</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
@@ -29667,7 +29667,7 @@
       </c>
       <c r="Q90" t="inlineStr">
         <is>
-          <t>40 + 10 + 85 (live REST 2026-10-17)</t>
+          <t>4 polygons, 1 per CA (live REST 2026-10-17)</t>
         </is>
       </c>
       <c r="R90" t="inlineStr">
@@ -29717,7 +29717,7 @@
       </c>
       <c r="AA90" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="AB90" t="inlineStr">
@@ -29832,7 +29832,7 @@
       </c>
       <c r="AX90" t="inlineStr">
         <is>
-          <t>A08. Context label. Evidence: live_rest.</t>
+          <t>A07. Four URLs expanded from the grouping template [inferred expansion]. Names the regulating CA so CH/GRCA refusals stay honest. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY90" t="inlineStr">
@@ -29919,7 +29919,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>grca_regulation_limits_waterloo_copy</t>
+          <t>hamilton_subwatersheds</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -29929,22 +29929,22 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>GRCA Regulation Limits (Region of Waterloo hosted copy)</t>
+          <t>Hamilton HCA / NPCA subwatersheds and watershed grades</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Grand River Conservation Authority (served by Region of Waterloo ITS-GIS)</t>
+          <t>City of Hamilton</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>https://utility.arcgis.com/usrsvcs/servers/7816f003cfd74d6591ccc5023a62b230/rest/services/_GRCA_Regulatory/MapServer/2</t>
+          <t>https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/HCA_Subwatersheds/FeatureServer | https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/NPCA_Subwatersheds/FeatureServer | https://services.arcgis.com/rYz782eMbySr2srL/arcgis/rest/services/Watershed_Grades/FeatureServer</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>West Hamilton / Flamborough (GRCA territory)</t>
+          <t>City of Hamilton</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -29959,7 +29959,7 @@
       </c>
       <c r="I91" t="inlineStr">
         <is>
-          <t>CA regulation polygons</t>
+          <t>subwatershed polygons</t>
         </is>
       </c>
       <c r="J91" t="inlineStr">
@@ -29969,7 +29969,7 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>REG_NUMBER | MU_LTIER</t>
+          <t/>
         </is>
       </c>
       <c r="L91" t="inlineStr">
@@ -29994,12 +29994,12 @@
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>ArcGIS MapServer</t>
+          <t>ArcGIS FeatureServer</t>
         </is>
       </c>
       <c r="Q91" t="inlineStr">
         <is>
-          <t>188 with MU_LTIER = CITY OF HAMILTON (live REST 2026-10-17)</t>
+          <t>40 + 10 + 85 (live REST 2026-10-17)</t>
         </is>
       </c>
       <c r="R91" t="inlineStr">
@@ -30049,7 +30049,7 @@
       </c>
       <c r="AA91" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="AB91" t="inlineStr">
@@ -30084,7 +30084,7 @@
       </c>
       <c r="AH91" t="inlineStr">
         <is>
-          <t>Third-party proxy | currency unknown | trial-pull only</t>
+          <t/>
         </is>
       </c>
       <c r="AI91" t="inlineStr">
@@ -30164,7 +30164,7 @@
       </c>
       <c r="AX91" t="inlineStr">
         <is>
-          <t>A10. Available via a Region of Waterloo hosted copy, to be trial-pulled. Distinct from GRCA-native maps.grandriver.ca Regulation Limit. Evidence: live_rest.</t>
+          <t>A08. Context label. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY91" t="inlineStr">
@@ -30251,7 +30251,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>conservation_halton_regulation_limit</t>
+          <t>grca_regulation_limits_waterloo_copy</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -30261,22 +30261,22 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Conservation Halton regulation limit (named gap)</t>
+          <t>GRCA Regulation Limits (Region of Waterloo hosted copy)</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Conservation Halton</t>
+          <t>Grand River Conservation Authority (served by Region of Waterloo ITS-GIS)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t/>
+          <t>https://utility.arcgis.com/usrsvcs/servers/7816f003cfd74d6591ccc5023a62b230/rest/services/_GRCA_Regulatory/MapServer/2</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>North Hamilton: Waterdown / Flamborough east</t>
+          <t>West Hamilton / Flamborough (GRCA territory)</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -30286,12 +30286,12 @@
       </c>
       <c r="H92" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>full</t>
         </is>
       </c>
       <c r="I92" t="inlineStr">
         <is>
-          <t>CA regulation polygons (not found)</t>
+          <t>CA regulation polygons</t>
         </is>
       </c>
       <c r="J92" t="inlineStr">
@@ -30301,7 +30301,7 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t/>
+          <t>REG_NUMBER | MU_LTIER</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
@@ -30321,52 +30321,52 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
+          <t>rest_bulk</t>
+        </is>
+      </c>
+      <c r="P92" t="inlineStr">
+        <is>
+          <t>ArcGIS MapServer</t>
+        </is>
+      </c>
+      <c r="Q92" t="inlineStr">
+        <is>
+          <t>188 with MU_LTIER = CITY OF HAMILTON (live REST 2026-10-17)</t>
+        </is>
+      </c>
+      <c r="R92" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U92" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V92" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="W92" t="inlineStr">
+        <is>
           <t>none</t>
         </is>
       </c>
-      <c r="P92" t="inlineStr">
-        <is>
-          <t>web map only (no open layer found)</t>
-        </is>
-      </c>
-      <c r="Q92" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
-      </c>
-      <c r="R92" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S92" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T92" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U92" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="V92" t="inlineStr">
-        <is>
-          <t>unclear</t>
-        </is>
-      </c>
-      <c r="W92" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
       <c r="X92" t="inlineStr">
         <is>
-          <t>inferred</t>
+          <t>authoritative</t>
         </is>
       </c>
       <c r="Y92" t="inlineStr">
@@ -30386,7 +30386,7 @@
       </c>
       <c r="AB92" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t/>
         </is>
       </c>
       <c r="AC92" t="inlineStr">
@@ -30401,7 +30401,7 @@
       </c>
       <c r="AE92" t="inlineStr">
         <is>
-          <t>not_found</t>
+          <t>candidate</t>
         </is>
       </c>
       <c r="AF92" t="inlineStr">
@@ -30416,7 +30416,7 @@
       </c>
       <c r="AH92" t="inlineStr">
         <is>
-          <t>not_found | named gap | no open REST endpoint</t>
+          <t>Third-party proxy | currency unknown | trial-pull only</t>
         </is>
       </c>
       <c r="AI92" t="inlineStr">
@@ -30496,7 +30496,7 @@
       </c>
       <c r="AX92" t="inlineStr">
         <is>
-          <t>A11. Conservation Halton has no open regulation layer found (2026-10-17 zero-result scan). Status: not_found / named gap. Do not invent coverage. Refuse not_in_coverage on CH-area parcels.</t>
+          <t>A10. Available via a Region of Waterloo hosted copy, to be trial-pulled. Distinct from GRCA-native maps.grandriver.ca Regulation Limit. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY92" t="inlineStr">
@@ -30583,7 +30583,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>lio_greenbelt_outer_boundary</t>
+          <t>conservation_halton_regulation_limit</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -30593,22 +30593,22 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Greenbelt Outer Boundary (LIO)</t>
+          <t>Conservation Halton regulation limit (named gap)</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Ontario MNR (LIO)</t>
+          <t>Conservation Halton</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open06/MapServer/17</t>
+          <t/>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>City of Hamilton bbox (1 polygon)</t>
+          <t>North Hamilton: Waterdown / Flamborough east</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -30618,12 +30618,12 @@
       </c>
       <c r="H93" t="inlineStr">
         <is>
-          <t>full</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="I93" t="inlineStr">
         <is>
-          <t>plan-area boundary</t>
+          <t>CA regulation polygons (not found)</t>
         </is>
       </c>
       <c r="J93" t="inlineStr">
@@ -30653,17 +30653,17 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>rest_bulk</t>
+          <t>none</t>
         </is>
       </c>
       <c r="P93" t="inlineStr">
         <is>
-          <t>ArcGIS MapServer</t>
+          <t>web map only (no open layer found)</t>
         </is>
       </c>
       <c r="Q93" t="inlineStr">
         <is>
-          <t>1 in Hamilton bbox (live REST bbox 2026-10-17)</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="R93" t="inlineStr">
@@ -30683,7 +30683,7 @@
       </c>
       <c r="U93" t="inlineStr">
         <is>
-          <t>Open Government Licence - Ontario [inferred; not re-read 2026-10-17]</t>
+          <t/>
         </is>
       </c>
       <c r="V93" t="inlineStr">
@@ -30698,7 +30698,7 @@
       </c>
       <c r="X93" t="inlineStr">
         <is>
-          <t>authoritative</t>
+          <t>inferred</t>
         </is>
       </c>
       <c r="Y93" t="inlineStr">
@@ -30713,12 +30713,12 @@
       </c>
       <c r="AA93" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="AB93" t="inlineStr">
         <is>
-          <t/>
+          <t>n/a</t>
         </is>
       </c>
       <c r="AC93" t="inlineStr">
@@ -30733,12 +30733,12 @@
       </c>
       <c r="AE93" t="inlineStr">
         <is>
-          <t>candidate</t>
+          <t>not_found</t>
         </is>
       </c>
       <c r="AF93" t="inlineStr">
         <is>
-          <t>basemap</t>
+          <t>constraint</t>
         </is>
       </c>
       <c r="AG93" t="inlineStr">
@@ -30748,7 +30748,7 @@
       </c>
       <c r="AH93" t="inlineStr">
         <is>
-          <t/>
+          <t>not_found | named gap | no open REST endpoint</t>
         </is>
       </c>
       <c r="AI93" t="inlineStr">
@@ -30828,7 +30828,7 @@
       </c>
       <c r="AX93" t="inlineStr">
         <is>
-          <t>A12. Nature-frame P1. Bbox count. Evidence: live_rest.</t>
+          <t>A11. Conservation Halton has no open regulation layer found (2026-10-17 zero-result scan). Status: not_found / named gap. Do not invent coverage. Refuse not_in_coverage on CH-area parcels.</t>
         </is>
       </c>
       <c r="AY93" t="inlineStr">
@@ -30853,7 +30853,7 @@
       </c>
       <c r="BC93" t="inlineStr">
         <is>
-          <t/>
+          <t>constraints</t>
         </is>
       </c>
       <c r="BD93" t="inlineStr">
@@ -30915,7 +30915,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>lio_natural_heritage_system</t>
+          <t>lio_greenbelt_outer_boundary</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -30925,7 +30925,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Natural Heritage System (LIO)</t>
+          <t>Greenbelt Outer Boundary (LIO)</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -30935,12 +30935,12 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open06/MapServer/22</t>
+          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open06/MapServer/17</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>City of Hamilton bbox</t>
+          <t>City of Hamilton bbox (1 polygon)</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -30955,7 +30955,7 @@
       </c>
       <c r="I94" t="inlineStr">
         <is>
-          <t>NHS polygons</t>
+          <t>plan-area boundary</t>
         </is>
       </c>
       <c r="J94" t="inlineStr">
@@ -30995,7 +30995,7 @@
       </c>
       <c r="Q94" t="inlineStr">
         <is>
-          <t>264 in Hamilton bbox (live REST bbox 2026-10-17)</t>
+          <t>1 in Hamilton bbox (live REST bbox 2026-10-17)</t>
         </is>
       </c>
       <c r="R94" t="inlineStr">
@@ -31045,7 +31045,7 @@
       </c>
       <c r="AA94" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="AB94" t="inlineStr">
@@ -31070,7 +31070,7 @@
       </c>
       <c r="AF94" t="inlineStr">
         <is>
-          <t>constraint</t>
+          <t>basemap</t>
         </is>
       </c>
       <c r="AG94" t="inlineStr">
@@ -31160,7 +31160,7 @@
       </c>
       <c r="AX94" t="inlineStr">
         <is>
-          <t>A13. Evidence: live_rest.</t>
+          <t>A12. Nature-frame P1. Bbox count. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY94" t="inlineStr">
@@ -31185,7 +31185,7 @@
       </c>
       <c r="BC94" t="inlineStr">
         <is>
-          <t>constraints</t>
+          <t/>
         </is>
       </c>
       <c r="BD94" t="inlineStr">
@@ -31247,7 +31247,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>lio_greenbelt_specialty_crop</t>
+          <t>lio_natural_heritage_system</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -31257,7 +31257,7 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Greenbelt Specialty Crop Area (LIO)</t>
+          <t>Natural Heritage System (LIO)</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -31267,7 +31267,7 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open06/MapServer/19</t>
+          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open06/MapServer/22</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
@@ -31287,7 +31287,7 @@
       </c>
       <c r="I95" t="inlineStr">
         <is>
-          <t>specialty-crop polygons</t>
+          <t>NHS polygons</t>
         </is>
       </c>
       <c r="J95" t="inlineStr">
@@ -31327,7 +31327,7 @@
       </c>
       <c r="Q95" t="inlineStr">
         <is>
-          <t>1 in Hamilton bbox (live REST bbox 2026-10-17)</t>
+          <t>264 in Hamilton bbox (live REST bbox 2026-10-17)</t>
         </is>
       </c>
       <c r="R95" t="inlineStr">
@@ -31377,7 +31377,7 @@
       </c>
       <c r="AA95" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="AB95" t="inlineStr">
@@ -31492,7 +31492,7 @@
       </c>
       <c r="AX95" t="inlineStr">
         <is>
-          <t>A14. Evidence: live_rest.</t>
+          <t>A13. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY95" t="inlineStr">
@@ -31517,7 +31517,7 @@
       </c>
       <c r="BC95" t="inlineStr">
         <is>
-          <t>land_use</t>
+          <t>constraints</t>
         </is>
       </c>
       <c r="BD95" t="inlineStr">
@@ -31579,7 +31579,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>lio_greenbelt_towns_villages</t>
+          <t>lio_greenbelt_specialty_crop</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -31589,7 +31589,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Greenbelt Towns and Villages (LIO)</t>
+          <t>Greenbelt Specialty Crop Area (LIO)</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -31599,7 +31599,7 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open06/MapServer/20</t>
+          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open06/MapServer/19</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
@@ -31619,7 +31619,7 @@
       </c>
       <c r="I96" t="inlineStr">
         <is>
-          <t>settlement polygons</t>
+          <t>specialty-crop polygons</t>
         </is>
       </c>
       <c r="J96" t="inlineStr">
@@ -31659,7 +31659,7 @@
       </c>
       <c r="Q96" t="inlineStr">
         <is>
-          <t>4 in Hamilton bbox (live REST bbox 2026-10-17)</t>
+          <t>1 in Hamilton bbox (live REST bbox 2026-10-17)</t>
         </is>
       </c>
       <c r="R96" t="inlineStr">
@@ -31734,7 +31734,7 @@
       </c>
       <c r="AF96" t="inlineStr">
         <is>
-          <t>basemap</t>
+          <t>constraint</t>
         </is>
       </c>
       <c r="AG96" t="inlineStr">
@@ -31824,7 +31824,7 @@
       </c>
       <c r="AX96" t="inlineStr">
         <is>
-          <t>A15. Evidence: live_rest.</t>
+          <t>A14. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY96" t="inlineStr">
@@ -31911,7 +31911,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>lio_greenbelt_hamlets</t>
+          <t>lio_greenbelt_towns_villages</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -31921,7 +31921,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Greenbelt Hamlets (LIO)</t>
+          <t>Greenbelt Towns and Villages (LIO)</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -31931,7 +31931,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open06/MapServer/16</t>
+          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open06/MapServer/20</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
@@ -31951,12 +31951,12 @@
       </c>
       <c r="I97" t="inlineStr">
         <is>
-          <t>hamlet points</t>
+          <t>settlement polygons</t>
         </is>
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>point_business</t>
+          <t>polygon_zone</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -31991,7 +31991,7 @@
       </c>
       <c r="Q97" t="inlineStr">
         <is>
-          <t>20 in Hamilton bbox (live REST bbox 2026-10-17)</t>
+          <t>4 in Hamilton bbox (live REST bbox 2026-10-17)</t>
         </is>
       </c>
       <c r="R97" t="inlineStr">
@@ -32156,7 +32156,7 @@
       </c>
       <c r="AX97" t="inlineStr">
         <is>
-          <t>A16. Evidence: live_rest.</t>
+          <t>A15. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY97" t="inlineStr">
@@ -32181,7 +32181,7 @@
       </c>
       <c r="BC97" t="inlineStr">
         <is>
-          <t/>
+          <t>land_use</t>
         </is>
       </c>
       <c r="BD97" t="inlineStr">
@@ -32243,7 +32243,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>lio_nep_area_boundary</t>
+          <t>lio_greenbelt_hamlets</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -32253,7 +32253,7 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Niagara Escarpment Plan Area boundary (LIO)</t>
+          <t>Greenbelt Hamlets (LIO)</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -32263,7 +32263,7 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open06/MapServer/25</t>
+          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open06/MapServer/16</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -32283,12 +32283,12 @@
       </c>
       <c r="I98" t="inlineStr">
         <is>
-          <t>plan-area boundary</t>
+          <t>hamlet points</t>
         </is>
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>polygon_zone</t>
+          <t>point_business</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -32323,7 +32323,7 @@
       </c>
       <c r="Q98" t="inlineStr">
         <is>
-          <t>1 in Hamilton bbox (live REST bbox 2026-10-17)</t>
+          <t>20 in Hamilton bbox (live REST bbox 2026-10-17)</t>
         </is>
       </c>
       <c r="R98" t="inlineStr">
@@ -32373,7 +32373,7 @@
       </c>
       <c r="AA98" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="AB98" t="inlineStr">
@@ -32488,7 +32488,7 @@
       </c>
       <c r="AX98" t="inlineStr">
         <is>
-          <t>A17. Nature-frame P1. Evidence: live_rest.</t>
+          <t>A16. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY98" t="inlineStr">
@@ -32575,7 +32575,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>lio_nep_policy_areas</t>
+          <t>lio_nep_area_boundary</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -32585,7 +32585,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Niagara Escarpment Plan Policy Areas (LIO)</t>
+          <t>Niagara Escarpment Plan Area boundary (LIO)</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -32595,7 +32595,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open06/MapServer/27</t>
+          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open06/MapServer/25</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
@@ -32615,7 +32615,7 @@
       </c>
       <c r="I99" t="inlineStr">
         <is>
-          <t>NEP policy polygons</t>
+          <t>plan-area boundary</t>
         </is>
       </c>
       <c r="J99" t="inlineStr">
@@ -32655,7 +32655,7 @@
       </c>
       <c r="Q99" t="inlineStr">
         <is>
-          <t>3 in Hamilton bbox (live REST bbox 2026-10-17)</t>
+          <t>1 in Hamilton bbox (live REST bbox 2026-10-17)</t>
         </is>
       </c>
       <c r="R99" t="inlineStr">
@@ -32705,7 +32705,7 @@
       </c>
       <c r="AA99" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="AB99" t="inlineStr">
@@ -32730,7 +32730,7 @@
       </c>
       <c r="AF99" t="inlineStr">
         <is>
-          <t>constraint</t>
+          <t>basemap</t>
         </is>
       </c>
       <c r="AG99" t="inlineStr">
@@ -32820,7 +32820,7 @@
       </c>
       <c r="AX99" t="inlineStr">
         <is>
-          <t>A18. Evidence: live_rest.</t>
+          <t>A17. Nature-frame P1. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY99" t="inlineStr">
@@ -32907,7 +32907,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>lio_nep_minor_urban_centres</t>
+          <t>lio_nep_policy_areas</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -32917,7 +32917,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Niagara Escarpment Plan Minor Urban Centres (LIO)</t>
+          <t>Niagara Escarpment Plan Policy Areas (LIO)</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -32927,7 +32927,7 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open06/MapServer/24</t>
+          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open06/MapServer/27</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
@@ -32947,7 +32947,7 @@
       </c>
       <c r="I100" t="inlineStr">
         <is>
-          <t>NEP settlement features</t>
+          <t>NEP policy polygons</t>
         </is>
       </c>
       <c r="J100" t="inlineStr">
@@ -32987,7 +32987,7 @@
       </c>
       <c r="Q100" t="inlineStr">
         <is>
-          <t>6 in Hamilton bbox (live REST bbox 2026-10-17)</t>
+          <t>3 in Hamilton bbox (live REST bbox 2026-10-17)</t>
         </is>
       </c>
       <c r="R100" t="inlineStr">
@@ -33062,7 +33062,7 @@
       </c>
       <c r="AF100" t="inlineStr">
         <is>
-          <t>basemap</t>
+          <t>constraint</t>
         </is>
       </c>
       <c r="AG100" t="inlineStr">
@@ -33152,7 +33152,7 @@
       </c>
       <c r="AX100" t="inlineStr">
         <is>
-          <t>A19. Evidence: live_rest.</t>
+          <t>A18. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY100" t="inlineStr">
@@ -33239,7 +33239,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>lio_wetlands</t>
+          <t>lio_nep_minor_urban_centres</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -33249,7 +33249,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Wetlands with significance (LIO provincial)</t>
+          <t>Niagara Escarpment Plan Minor Urban Centres (LIO)</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -33259,7 +33259,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open01/MapServer/15</t>
+          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open06/MapServer/24</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
@@ -33279,7 +33279,7 @@
       </c>
       <c r="I101" t="inlineStr">
         <is>
-          <t>wetland polygons</t>
+          <t>NEP settlement features</t>
         </is>
       </c>
       <c r="J101" t="inlineStr">
@@ -33319,7 +33319,7 @@
       </c>
       <c r="Q101" t="inlineStr">
         <is>
-          <t>5718 in Hamilton bbox (live REST bbox 2026-10-17)</t>
+          <t>6 in Hamilton bbox (live REST bbox 2026-10-17)</t>
         </is>
       </c>
       <c r="R101" t="inlineStr">
@@ -33394,7 +33394,7 @@
       </c>
       <c r="AF101" t="inlineStr">
         <is>
-          <t>constraint</t>
+          <t>basemap</t>
         </is>
       </c>
       <c r="AG101" t="inlineStr">
@@ -33484,7 +33484,7 @@
       </c>
       <c r="AX101" t="inlineStr">
         <is>
-          <t>A20. Prefer hamilton_wetlands inside the city. Evidence: live_rest.</t>
+          <t>A19. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY101" t="inlineStr">
@@ -33509,7 +33509,7 @@
       </c>
       <c r="BC101" t="inlineStr">
         <is>
-          <t>constraints</t>
+          <t/>
         </is>
       </c>
       <c r="BD101" t="inlineStr">
@@ -33571,7 +33571,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>lio_ansi</t>
+          <t>lio_wetlands</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -33581,7 +33581,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Areas of Natural and Scientific Interest (LIO)</t>
+          <t>Wetlands with significance (LIO provincial)</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -33591,7 +33591,7 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open05/MapServer/3</t>
+          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open01/MapServer/15</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
@@ -33611,7 +33611,7 @@
       </c>
       <c r="I102" t="inlineStr">
         <is>
-          <t>ANSI polygons</t>
+          <t>wetland polygons</t>
         </is>
       </c>
       <c r="J102" t="inlineStr">
@@ -33621,7 +33621,7 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>ANSI_NAME | ANSI_SIGNIFICANCE</t>
+          <t/>
         </is>
       </c>
       <c r="L102" t="inlineStr">
@@ -33651,7 +33651,7 @@
       </c>
       <c r="Q102" t="inlineStr">
         <is>
-          <t>71 in Hamilton bbox (live REST bbox 2026-10-17)</t>
+          <t>5718 in Hamilton bbox (live REST bbox 2026-10-17)</t>
         </is>
       </c>
       <c r="R102" t="inlineStr">
@@ -33681,7 +33681,7 @@
       </c>
       <c r="W102" t="inlineStr">
         <is>
-          <t>none (LANDOWNER_CONTACT_FLG is a field name only)</t>
+          <t>none</t>
         </is>
       </c>
       <c r="X102" t="inlineStr">
@@ -33701,7 +33701,7 @@
       </c>
       <c r="AA102" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="AB102" t="inlineStr">
@@ -33816,7 +33816,7 @@
       </c>
       <c r="AX102" t="inlineStr">
         <is>
-          <t>A21. Owner-like field name LANDOWNER_CONTACT_FLG recorded; no values. Evidence: live_rest.</t>
+          <t>A20. Prefer hamilton_wetlands inside the city. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY102" t="inlineStr">
@@ -33903,7 +33903,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>lio_wooded_areas</t>
+          <t>lio_ansi</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -33913,7 +33913,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Wooded Areas (LIO)</t>
+          <t>Areas of Natural and Scientific Interest (LIO)</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -33923,7 +33923,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open07/MapServer/29</t>
+          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open05/MapServer/3</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
@@ -33943,7 +33943,7 @@
       </c>
       <c r="I103" t="inlineStr">
         <is>
-          <t>wooded-area polygons</t>
+          <t>ANSI polygons</t>
         </is>
       </c>
       <c r="J103" t="inlineStr">
@@ -33953,7 +33953,7 @@
       </c>
       <c r="K103" t="inlineStr">
         <is>
-          <t/>
+          <t>ANSI_NAME | ANSI_SIGNIFICANCE</t>
         </is>
       </c>
       <c r="L103" t="inlineStr">
@@ -33983,7 +33983,7 @@
       </c>
       <c r="Q103" t="inlineStr">
         <is>
-          <t>7483 in Hamilton bbox (live REST bbox 2026-10-17)</t>
+          <t>71 in Hamilton bbox (live REST bbox 2026-10-17)</t>
         </is>
       </c>
       <c r="R103" t="inlineStr">
@@ -34013,7 +34013,7 @@
       </c>
       <c r="W103" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>none (LANDOWNER_CONTACT_FLG is a field name only)</t>
         </is>
       </c>
       <c r="X103" t="inlineStr">
@@ -34033,7 +34033,7 @@
       </c>
       <c r="AA103" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="AB103" t="inlineStr">
@@ -34058,7 +34058,7 @@
       </c>
       <c r="AF103" t="inlineStr">
         <is>
-          <t>basemap</t>
+          <t>constraint</t>
         </is>
       </c>
       <c r="AG103" t="inlineStr">
@@ -34148,7 +34148,7 @@
       </c>
       <c r="AX103" t="inlineStr">
         <is>
-          <t>A22. Nature-frame P1. Evidence: live_rest.</t>
+          <t>A21. Owner-like field name LANDOWNER_CONTACT_FLG recorded; no values. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY103" t="inlineStr">
@@ -34173,7 +34173,7 @@
       </c>
       <c r="BC103" t="inlineStr">
         <is>
-          <t/>
+          <t>constraints</t>
         </is>
       </c>
       <c r="BD103" t="inlineStr">
@@ -34235,7 +34235,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>lio_provincial_parks</t>
+          <t>lio_wooded_areas</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -34245,7 +34245,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Provincial parks regulated (LIO)</t>
+          <t>Wooded Areas (LIO)</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -34255,7 +34255,7 @@
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open03/MapServer/4</t>
+          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open07/MapServer/29</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
@@ -34275,7 +34275,7 @@
       </c>
       <c r="I104" t="inlineStr">
         <is>
-          <t>provincial park polygons</t>
+          <t>wooded-area polygons</t>
         </is>
       </c>
       <c r="J104" t="inlineStr">
@@ -34315,7 +34315,7 @@
       </c>
       <c r="Q104" t="inlineStr">
         <is>
-          <t>1 in Hamilton bbox (live REST bbox 2026-10-17)</t>
+          <t>7483 in Hamilton bbox (live REST bbox 2026-10-17)</t>
         </is>
       </c>
       <c r="R104" t="inlineStr">
@@ -34365,7 +34365,7 @@
       </c>
       <c r="AA104" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="AB104" t="inlineStr">
@@ -34480,7 +34480,7 @@
       </c>
       <c r="AX104" t="inlineStr">
         <is>
-          <t>A23. Evidence: live_rest.</t>
+          <t>A22. Nature-frame P1. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY104" t="inlineStr">
@@ -34567,7 +34567,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>lio_conservation_authority_admin</t>
+          <t>lio_provincial_parks</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -34577,7 +34577,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Conservation Authority administrative areas (LIO)</t>
+          <t>Provincial parks regulated (LIO)</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -34587,7 +34587,7 @@
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open03/MapServer/11</t>
+          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open03/MapServer/4</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
@@ -34607,7 +34607,7 @@
       </c>
       <c r="I105" t="inlineStr">
         <is>
-          <t>CA administrative polygons</t>
+          <t>provincial park polygons</t>
         </is>
       </c>
       <c r="J105" t="inlineStr">
@@ -34647,7 +34647,7 @@
       </c>
       <c r="Q105" t="inlineStr">
         <is>
-          <t>4 in Hamilton bbox (live REST bbox 2026-10-17)</t>
+          <t>1 in Hamilton bbox (live REST bbox 2026-10-17)</t>
         </is>
       </c>
       <c r="R105" t="inlineStr">
@@ -34697,7 +34697,7 @@
       </c>
       <c r="AA105" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="AB105" t="inlineStr">
@@ -34722,7 +34722,7 @@
       </c>
       <c r="AF105" t="inlineStr">
         <is>
-          <t>constraint</t>
+          <t>basemap</t>
         </is>
       </c>
       <c r="AG105" t="inlineStr">
@@ -34812,7 +34812,7 @@
       </c>
       <c r="AX105" t="inlineStr">
         <is>
-          <t>A24. Evidence: live_rest.</t>
+          <t>A23. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY105" t="inlineStr">
@@ -34899,7 +34899,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>lio_municipal_boundary</t>
+          <t>lio_conservation_authority_admin</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -34909,7 +34909,7 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Municipal boundary (LIO, MUNID / ASSESSMENT_CODE)</t>
+          <t>Conservation Authority administrative areas (LIO)</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
@@ -34919,7 +34919,7 @@
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open03/MapServer/14</t>
+          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open03/MapServer/11</t>
         </is>
       </c>
       <c r="F106" t="inlineStr">
@@ -34939,7 +34939,7 @@
       </c>
       <c r="I106" t="inlineStr">
         <is>
-          <t>municipal boundary polygons</t>
+          <t>CA administrative polygons</t>
         </is>
       </c>
       <c r="J106" t="inlineStr">
@@ -34949,7 +34949,7 @@
       </c>
       <c r="K106" t="inlineStr">
         <is>
-          <t>MUNID | ASSESSMENT_CODE</t>
+          <t/>
         </is>
       </c>
       <c r="L106" t="inlineStr">
@@ -34979,7 +34979,7 @@
       </c>
       <c r="Q106" t="inlineStr">
         <is>
-          <t>16 in Hamilton bbox (live REST bbox 2026-10-17)</t>
+          <t>4 in Hamilton bbox (live REST bbox 2026-10-17)</t>
         </is>
       </c>
       <c r="R106" t="inlineStr">
@@ -35029,7 +35029,7 @@
       </c>
       <c r="AA106" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="AB106" t="inlineStr">
@@ -35054,7 +35054,7 @@
       </c>
       <c r="AF106" t="inlineStr">
         <is>
-          <t>unit_spine</t>
+          <t>constraint</t>
         </is>
       </c>
       <c r="AG106" t="inlineStr">
@@ -35144,7 +35144,7 @@
       </c>
       <c r="AX106" t="inlineStr">
         <is>
-          <t>A25. ASSESSMENT_CODE can validate ARN prefix 2518. Evidence: live_rest.</t>
+          <t>A24. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY106" t="inlineStr">
@@ -35169,7 +35169,7 @@
       </c>
       <c r="BC106" t="inlineStr">
         <is>
-          <t>identity</t>
+          <t/>
         </is>
       </c>
       <c r="BD106" t="inlineStr">
@@ -35231,7 +35231,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>lio_ontario_trails_network</t>
+          <t>lio_municipal_boundary</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -35241,7 +35241,7 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Ontario Trails Network segments (LIO)</t>
+          <t>Municipal boundary (LIO, MUNID / ASSESSMENT_CODE)</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -35251,7 +35251,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open04/MapServer/19</t>
+          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open03/MapServer/14</t>
         </is>
       </c>
       <c r="F107" t="inlineStr">
@@ -35271,7 +35271,7 @@
       </c>
       <c r="I107" t="inlineStr">
         <is>
-          <t>trail segments</t>
+          <t>municipal boundary polygons</t>
         </is>
       </c>
       <c r="J107" t="inlineStr">
@@ -35281,7 +35281,7 @@
       </c>
       <c r="K107" t="inlineStr">
         <is>
-          <t/>
+          <t>MUNID | ASSESSMENT_CODE</t>
         </is>
       </c>
       <c r="L107" t="inlineStr">
@@ -35311,7 +35311,7 @@
       </c>
       <c r="Q107" t="inlineStr">
         <is>
-          <t>628 in Hamilton bbox (live REST bbox 2026-10-17)</t>
+          <t>16 in Hamilton bbox (live REST bbox 2026-10-17)</t>
         </is>
       </c>
       <c r="R107" t="inlineStr">
@@ -35361,7 +35361,7 @@
       </c>
       <c r="AA107" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="AB107" t="inlineStr">
@@ -35386,7 +35386,7 @@
       </c>
       <c r="AF107" t="inlineStr">
         <is>
-          <t>basemap</t>
+          <t>unit_spine</t>
         </is>
       </c>
       <c r="AG107" t="inlineStr">
@@ -35476,7 +35476,7 @@
       </c>
       <c r="AX107" t="inlineStr">
         <is>
-          <t>A26. Evidence: live_rest.</t>
+          <t>A25. ASSESSMENT_CODE can validate ARN prefix 2518. Evidence: live_rest.</t>
         </is>
       </c>
       <c r="AY107" t="inlineStr">
@@ -35501,7 +35501,7 @@
       </c>
       <c r="BC107" t="inlineStr">
         <is>
-          <t/>
+          <t>identity</t>
         </is>
       </c>
       <c r="BD107" t="inlineStr">
@@ -35563,330 +35563,662 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
+          <t>lio_ontario_trails_network</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Ontario Trails Network segments (LIO)</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Ontario MNR (LIO)</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>https://ws.lioservices.lrc.gov.on.ca/arcgis2/rest/services/LIO_OPEN_DATA/LIO_Open04/MapServer/19</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>City of Hamilton bbox</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>ON-Hamilton</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>full</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>trail segments</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>polygon_zone</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O108" t="inlineStr">
+        <is>
+          <t>rest_bulk</t>
+        </is>
+      </c>
+      <c r="P108" t="inlineStr">
+        <is>
+          <t>ArcGIS MapServer</t>
+        </is>
+      </c>
+      <c r="Q108" t="inlineStr">
+        <is>
+          <t>628 in Hamilton bbox (live REST bbox 2026-10-17)</t>
+        </is>
+      </c>
+      <c r="R108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>Open Government Licence - Ontario [inferred; not re-read 2026-10-17]</t>
+        </is>
+      </c>
+      <c r="V108" t="inlineStr">
+        <is>
+          <t>unclear</t>
+        </is>
+      </c>
+      <c r="W108" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="X108" t="inlineStr">
+        <is>
+          <t>authoritative</t>
+        </is>
+      </c>
+      <c r="Y108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA108" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="AB108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC108" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="AD108" t="inlineStr">
+        <is>
+          <t>not_started</t>
+        </is>
+      </c>
+      <c r="AE108" t="inlineStr">
+        <is>
+          <t>candidate</t>
+        </is>
+      </c>
+      <c r="AF108" t="inlineStr">
+        <is>
+          <t>basemap</t>
+        </is>
+      </c>
+      <c r="AG108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AH108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AI108" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="AJ108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AK108" t="inlineStr">
+        <is>
+          <t>Hamilton grouping analysis 2026-10-17</t>
+        </is>
+      </c>
+      <c r="AL108" t="inlineStr">
+        <is>
+          <t>niagaraassembly/heavymap</t>
+        </is>
+      </c>
+      <c r="AM108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AN108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AP108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AQ108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AR108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AS108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AT108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AU108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AV108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AW108" t="inlineStr">
+        <is>
+          <t>missing</t>
+        </is>
+      </c>
+      <c r="AX108" t="inlineStr">
+        <is>
+          <t>A26. Evidence: live_rest.</t>
+        </is>
+      </c>
+      <c r="AY108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AZ108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BA108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BB108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BC108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BD108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BE108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BF108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BG108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BH108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BI108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BJ108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BK108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BL108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BM108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BN108" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
           <t>hca_trails</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="C108" t="inlineStr">
+      <c r="B109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
         <is>
           <t>HCA Trails</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr">
+      <c r="D109" t="inlineStr">
         <is>
           <t>Hamilton Conservation Authority</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr">
+      <c r="E109" t="inlineStr">
         <is>
           <t>https://services1.arcgis.com/d0ZCwU7eGKVeNiEE/arcgis/rest/services/HCA_Trails/FeatureServer/4</t>
         </is>
       </c>
-      <c r="F108" t="inlineStr">
+      <c r="F109" t="inlineStr">
         <is>
           <t>Hamilton-area watersheds</t>
         </is>
       </c>
-      <c r="G108" t="inlineStr">
+      <c r="G109" t="inlineStr">
         <is>
           <t>ON-Hamilton</t>
         </is>
       </c>
-      <c r="H108" t="inlineStr">
+      <c r="H109" t="inlineStr">
         <is>
           <t>full</t>
         </is>
       </c>
-      <c r="I108" t="inlineStr">
+      <c r="I109" t="inlineStr">
         <is>
           <t>HCA trail lines</t>
         </is>
       </c>
-      <c r="J108" t="inlineStr">
+      <c r="J109" t="inlineStr">
         <is>
           <t>polygon_zone</t>
         </is>
       </c>
-      <c r="K108" t="inlineStr">
+      <c r="K109" t="inlineStr">
         <is>
           <t>Trail_Name | BTC_Name | Conservation_Area</t>
         </is>
       </c>
-      <c r="L108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="M108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="N108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="O108" t="inlineStr">
+      <c r="L109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="O109" t="inlineStr">
         <is>
           <t>rest_bulk</t>
         </is>
       </c>
-      <c r="P108" t="inlineStr">
+      <c r="P109" t="inlineStr">
         <is>
           <t>ArcGIS FeatureServer</t>
         </is>
       </c>
-      <c r="Q108" t="inlineStr">
+      <c r="Q109" t="inlineStr">
         <is>
           <t>count not in the grouping CSV; live REST 2026-10-17</t>
         </is>
       </c>
-      <c r="R108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="S108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="T108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="U108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="V108" t="inlineStr">
+      <c r="R109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="V109" t="inlineStr">
         <is>
           <t>unclear</t>
         </is>
       </c>
-      <c r="W108" t="inlineStr">
+      <c r="W109" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
-      <c r="X108" t="inlineStr">
+      <c r="X109" t="inlineStr">
         <is>
           <t>authoritative</t>
         </is>
       </c>
-      <c r="Y108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="Z108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AA108" t="inlineStr">
+      <c r="Y109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="Z109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AA109" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
       </c>
-      <c r="AB108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AC108" t="inlineStr">
+      <c r="AB109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AC109" t="inlineStr">
         <is>
           <t>not_started</t>
         </is>
       </c>
-      <c r="AD108" t="inlineStr">
+      <c r="AD109" t="inlineStr">
         <is>
           <t>not_started</t>
         </is>
       </c>
-      <c r="AE108" t="inlineStr">
+      <c r="AE109" t="inlineStr">
         <is>
           <t>candidate</t>
         </is>
       </c>
-      <c r="AF108" t="inlineStr">
+      <c r="AF109" t="inlineStr">
         <is>
           <t>basemap</t>
         </is>
       </c>
-      <c r="AG108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AH108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AI108" t="inlineStr">
+      <c r="AG109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AH109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AI109" t="inlineStr">
         <is>
           <t>2026-10-17</t>
         </is>
       </c>
-      <c r="AJ108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AK108" t="inlineStr">
+      <c r="AJ109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AK109" t="inlineStr">
         <is>
           <t>Hamilton grouping analysis 2026-10-17</t>
         </is>
       </c>
-      <c r="AL108" t="inlineStr">
+      <c r="AL109" t="inlineStr">
         <is>
           <t>niagaraassembly/heavymap</t>
         </is>
       </c>
-      <c r="AM108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AN108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AO108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AP108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AQ108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AR108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AS108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AT108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AU108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AV108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AW108" t="inlineStr">
+      <c r="AM109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AN109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AO109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AP109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AQ109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AR109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AS109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AT109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AU109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AV109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AW109" t="inlineStr">
         <is>
           <t>missing</t>
         </is>
       </c>
-      <c r="AX108" t="inlineStr">
+      <c r="AX109" t="inlineStr">
         <is>
           <t>A27. Re-admitted from reviewed_not_relevant. Ownership is a field name only. Evidence: live_rest.</t>
         </is>
       </c>
-      <c r="AY108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="AZ108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BA108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BB108" t="inlineStr">
+      <c r="AY109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="AZ109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BA109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BB109" t="inlineStr">
         <is>
           <t>contextual_only</t>
         </is>
       </c>
-      <c r="BC108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BD108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BE108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BF108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BG108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BH108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BI108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BJ108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BK108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BL108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BM108" t="inlineStr">
-        <is>
-          <t/>
-        </is>
-      </c>
-      <c r="BN108" t="inlineStr">
+      <c r="BC109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BD109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BE109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BF109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BG109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BH109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BI109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BJ109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BK109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BL109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BM109" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="BN109" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>